<commit_message>
Anonymize steward references (Rob -> Steward) in workbook + screenshots
</commit_message>
<xml_diff>
--- a/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
+++ b/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
@@ -962,7 +962,7 @@
       </c>
       <c r="D5" s="9" t="inlineStr">
         <is>
-          <t>Rob</t>
+          <t>Steward</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1004,7 +1004,7 @@
       </c>
       <c r="D6" s="9" t="inlineStr">
         <is>
-          <t>Rob</t>
+          <t>Steward</t>
         </is>
       </c>
       <c r="E6" s="9" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>Rob</t>
+          <t>Steward</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
@@ -2395,7 +2395,7 @@
     <row r="8">
       <c r="B8" s="23" t="inlineStr">
         <is>
-          <t>Rob</t>
+          <t>Steward</t>
         </is>
       </c>
       <c r="C8" s="26" t="n">

</xml_diff>

<commit_message>
mindsheets: two variants to isolate the Numbers recalculation behaviour
</commit_message>
<xml_diff>
--- a/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
+++ b/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
@@ -986,11 +986,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="8816042"/>
-        <c:axId val="7535287"/>
+        <c:axId val="76829479"/>
+        <c:axId val="62711170"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="8816042"/>
+        <c:axId val="76829479"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1023,7 +1023,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="7535287"/>
+        <c:crossAx val="62711170"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1031,7 +1031,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="7535287"/>
+        <c:axId val="62711170"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1074,7 +1074,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="8816042"/>
+        <c:crossAx val="76829479"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>

<commit_message>
mindsheets: real human testing log incl. the Numbers failure
</commit_message>
<xml_diff>
--- a/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
+++ b/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="115">
   <si>
     <t xml:space="preserve">BATTLE OF THE MINDS</t>
   </si>
@@ -244,10 +244,67 @@
     <t xml:space="preserve">Pass?</t>
   </si>
   <si>
+    <t xml:space="preserve">Recommendation excludes an event with no attempts left</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next Best Move D7 (Mindsheets Left): 2 -&gt; 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D14 switches to 'Calm before the Storm'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calm before the Storm (Excel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV reacts correctly to a lower spread</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D7 back to 2; G7 (Mindsheets sigma): 4.04 -&gt; 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I7 drops 0.97 -&gt; ~0.03; verdict 'low return'; D14 -&gt; Calm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as expected (Excel)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-app check: Apple Numbers, first build</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open build without cached values in Numbers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALL CELLS BLANK - Numbers does not recalculate imported formulas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-app check: Apple Numbers, after fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open build with fullCalcOnLoad + baked-in values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values shown AND live recalculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values shown; recalculation only after editing the cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARTIAL</t>
+  </si>
+  <si>
     <t xml:space="preserve">New submission totals correctly</t>
   </si>
   <si>
-    <t xml:space="preserve">F14=9; G14=8; H14=7</t>
+    <t xml:space="preserve">Submissions F14=9; G14=8; H14=7</t>
   </si>
   <si>
     <t xml:space="preserve">I14 = 24; Grade = Strong</t>
@@ -256,22 +313,7 @@
     <t xml:space="preserve">24; Strong</t>
   </si>
   <si>
-    <t xml:space="preserve">Pass</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reward pool splits &amp; dampens sybil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D5 = 3.0; C11 (SybilFarm Minds) = 12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TOTAL payout = 3.0000; SybilFarm &lt; Rob</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3.0000; 0.4686 &lt; 0.8609</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status: Ready — both test cases run by the human steward and passed.</t>
+    <t xml:space="preserve">Status: Ready — in Microsoft Excel and LibreOffice Calc, verified by the human steward. Apple Numbers displays every value but does not re-evaluate imported formulas until a cell is edited; that is a Numbers import behaviour, not a formula error, and it is listed above as test 3 (FAIL) and test 4 (PARTIAL) rather than omitted.</t>
   </si>
   <si>
     <t xml:space="preserve">NEXT BEST MOVE  ·  where should the next attempt go?</t>
@@ -986,11 +1028,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="76829479"/>
-        <c:axId val="62711170"/>
+        <c:axId val="19912915"/>
+        <c:axId val="82700268"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="76829479"/>
+        <c:axId val="19912915"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1023,7 +1065,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62711170"/>
+        <c:crossAx val="82700268"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1031,7 +1073,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62711170"/>
+        <c:axId val="82700268"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1074,7 +1116,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="76829479"/>
+        <c:crossAx val="19912915"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3170,14 +3212,15 @@
     <tabColor rgb="FF6B7280"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:G9"/>
+  <dimension ref="B2:G12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="9"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3250,9 +3293,69 @@
         <v>76</v>
       </c>
     </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B8" s="33" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="34" t="s">
+        <v>81</v>
+      </c>
+      <c r="D8" s="34" t="s">
+        <v>82</v>
+      </c>
+      <c r="E8" s="34" t="s">
+        <v>83</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>85</v>
+      </c>
+    </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="35" t="s">
-        <v>81</v>
+      <c r="B9" s="33" t="n">
+        <v>4</v>
+      </c>
+      <c r="C9" s="34" t="s">
+        <v>86</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>87</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>88</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>89</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B10" s="33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C10" s="34" t="s">
+        <v>91</v>
+      </c>
+      <c r="D10" s="34" t="s">
+        <v>92</v>
+      </c>
+      <c r="E10" s="34" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B12" s="35" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -3289,12 +3392,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>83</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3302,39 +3405,39 @@
         <v>19</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>84</v>
+        <v>98</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>86</v>
+        <v>100</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>88</v>
+        <v>102</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>89</v>
+        <v>103</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>28</v>
@@ -3374,7 +3477,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="34" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>25</v>
@@ -3494,7 +3597,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="34" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>26</v>
@@ -3534,7 +3637,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="34" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>26</v>
@@ -3574,7 +3677,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="34" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>26</v>
@@ -3614,7 +3717,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
       <c r="D14" s="41" t="str">
         <f aca="false">INDEX($B$6:$B$12,MATCH(MAX($K$6:$K$12),$K$6:$K$12,0))</f>
@@ -3623,7 +3726,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="42" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="C15" s="42"/>
       <c r="D15" s="42"/>

</xml_diff>

<commit_message>
mindsheets: real verified scores, fictional demo minds, best-per-event fix (SUMIFS -> SUMPRODUCT/MAX), independent 79-cell verifier
</commit_message>
<xml_diff>
--- a/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
+++ b/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc"/>
+  <fileVersion appName="Calc" lowestEdited="4"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="123">
   <si>
     <t xml:space="preserve">BATTLE OF THE MINDS</t>
   </si>
@@ -103,34 +103,46 @@
     <t xml:space="preserve">Grade</t>
   </si>
   <si>
+    <t xml:space="preserve">calc</t>
+  </si>
+  <si>
     <t xml:space="preserve">(event list — used by dropdown)</t>
   </si>
   <si>
     <t xml:space="preserve">NeoBerlin</t>
   </si>
   <si>
+    <t xml:space="preserve">Rob (human steward)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Special Skills using X</t>
+  </si>
+  <si>
     <t xml:space="preserve">More Minds are better than one Mind: Research Quest</t>
   </si>
   <si>
     <t xml:space="preserve">Cross Word Puzzle</t>
   </si>
   <si>
+    <t xml:space="preserve">Calm before the Storm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AstroMesh: Minds &amp; MCP Mashup Challenge</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minds Building Chatbots Challenge</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mindsheets Masterpiece and Debugging</t>
   </si>
   <si>
-    <t xml:space="preserve">Calm before the Storm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minty</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nip0r</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VARgentina</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Michael</t>
+    <t xml:space="preserve">Demo-Alpha</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(fictional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demo-Beta</t>
   </si>
   <si>
     <t xml:space="preserve">LEADERBOARD  ·  overall = sum of best submission per event</t>
@@ -139,19 +151,28 @@
     <t xml:space="preserve">Rank</t>
   </si>
   <si>
+    <t xml:space="preserve">X-Skill</t>
+  </si>
+  <si>
     <t xml:space="preserve">Research</t>
   </si>
   <si>
+    <t xml:space="preserve">Crossword</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AstroMesh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chatbots</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mindsheets</t>
   </si>
   <si>
-    <t xml:space="preserve">Crossword</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Overall /120</t>
+    <t xml:space="preserve">Overall /210</t>
   </si>
   <si>
     <t xml:space="preserve">Medal</t>
@@ -166,7 +187,7 @@
     <t xml:space="preserve">LEADER</t>
   </si>
   <si>
-    <t xml:space="preserve">TOP OVERALL /120</t>
+    <t xml:space="preserve">TOP OVERALL /210</t>
   </si>
   <si>
     <t xml:space="preserve">NEOBERLIN OVERALL</t>
@@ -208,7 +229,13 @@
     <t xml:space="preserve">Payout (ETH)</t>
   </si>
   <si>
-    <t xml:space="preserve">SybilFarm</t>
+    <t xml:space="preserve">(fictional) A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(fictional) B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SybilFarm (illustrative)</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -319,7 +346,7 @@
     <t xml:space="preserve">NEXT BEST MOVE  ·  where should the next attempt go?</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected value of ONE more attempt, per event. Only light-blue cells are inputs. mu = average of the last two scores (steward's choice); sigma = spread of all scores so far.</t>
+    <t xml:space="preserve">Expected value of ONE more attempt, per event. Best/Left/n come straight from the tournament API (GET /api/compete/puzzles and /submissions/me) on 2026-07-28. Only light-blue cells are inputs. mu = average of the last two scores (steward's choice); sigma = spread of all scores so far.</t>
   </si>
   <si>
     <t xml:space="preserve">Best</t>
@@ -355,16 +382,13 @@
     <t xml:space="preserve">More Minds are better than one</t>
   </si>
   <si>
+    <t xml:space="preserve">AstroMesh: Minds &amp; MCP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minds Building Chatbots</t>
+  </si>
+  <si>
     <t xml:space="preserve">Mindsheets Masterpiece</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minds Building Chatbots</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AstroMesh: Minds &amp; MCP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Special Skills using X</t>
   </si>
   <si>
     <t xml:space="preserve">RECOMMENDATION</t>
@@ -913,7 +937,7 @@
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Overall standings /120</a:t>
+              <a:t>Overall standings /210</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -999,10 +1023,10 @@
                   <c:v>NeoBerlin</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>Minty</c:v>
+                  <c:v>Demo-Alpha</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>VARgentina</c:v>
+                  <c:v>Demo-Beta</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1014,13 +1038,13 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="3"/>
                 <c:pt idx="0">
-                  <c:v>81</c:v>
+                  <c:v>186</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>108</c:v>
+                  <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>50</c:v>
+                  <c:v>43</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1028,11 +1052,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="19912915"/>
-        <c:axId val="82700268"/>
+        <c:axId val="50949338"/>
+        <c:axId val="45396134"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="19912915"/>
+        <c:axId val="50949338"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1065,7 +1089,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="82700268"/>
+        <c:crossAx val="45396134"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1073,7 +1097,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="82700268"/>
+        <c:axId val="45396134"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1116,7 +1140,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19912915"/>
+        <c:crossAx val="50949338"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1738,8 +1762,11 @@
       <c r="J4" s="6" t="s">
         <v>24</v>
       </c>
+      <c r="K4" s="7" t="s">
+        <v>25</v>
+      </c>
       <c r="M4" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1747,13 +1774,13 @@
         <v>1</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E5" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F5" s="10" t="n">
         <v>9</v>
@@ -1762,18 +1789,22 @@
         <v>9</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="I5" s="11" t="n">
         <f aca="false">IF(COUNT(F5:H5)=0,"",SUM(F5:H5))</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="J5" s="11" t="str">
         <f aca="false">IF(I5="","",IF(I5&gt;=27,"★ Elite",IF(I5&gt;=21,"Strong",IF(I5&gt;=15,"Fair","Weak"))))</f>
         <v>★ Elite</v>
       </c>
+      <c r="K5" s="12" t="n">
+        <f aca="false">IF(I5="",0,I5)</f>
+        <v>28</v>
+      </c>
       <c r="M5" s="12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1781,22 +1812,22 @@
         <v>2</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F6" s="10" t="n">
         <v>9</v>
       </c>
       <c r="G6" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="H6" s="10" t="n">
         <v>10</v>
-      </c>
-      <c r="H6" s="10" t="n">
-        <v>9</v>
       </c>
       <c r="I6" s="11" t="n">
         <f aca="false">IF(COUNT(F6:H6)=0,"",SUM(F6:H6))</f>
@@ -1806,8 +1837,12 @@
         <f aca="false">IF(I6="","",IF(I6&gt;=27,"★ Elite",IF(I6&gt;=21,"Strong",IF(I6&gt;=15,"Fair","Weak"))))</f>
         <v>★ Elite</v>
       </c>
+      <c r="K6" s="12" t="n">
+        <f aca="false">IF(I6="",0,I6)</f>
+        <v>28</v>
+      </c>
       <c r="M6" s="12" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1815,13 +1850,13 @@
         <v>3</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>9</v>
@@ -1830,18 +1865,22 @@
         <v>9</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="I7" s="11" t="n">
         <f aca="false">IF(COUNT(F7:H7)=0,"",SUM(F7:H7))</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="J7" s="11" t="str">
         <f aca="false">IF(I7="","",IF(I7&gt;=27,"★ Elite",IF(I7&gt;=21,"Strong",IF(I7&gt;=15,"Fair","Weak"))))</f>
-        <v>Strong</v>
+        <v>★ Elite</v>
+      </c>
+      <c r="K7" s="12" t="n">
+        <f aca="false">IF(I7="",0,I7)</f>
+        <v>27</v>
       </c>
       <c r="M7" s="12" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1849,33 +1888,37 @@
         <v>4</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D8" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="9" t="s">
         <v>32</v>
-      </c>
-      <c r="E8" s="9" t="s">
-        <v>27</v>
       </c>
       <c r="F8" s="10" t="n">
         <v>9</v>
       </c>
       <c r="G8" s="10" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="H8" s="10" t="n">
         <v>9</v>
       </c>
       <c r="I8" s="11" t="n">
         <f aca="false">IF(COUNT(F8:H8)=0,"",SUM(F8:H8))</f>
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="J8" s="11" t="str">
         <f aca="false">IF(I8="","",IF(I8&gt;=27,"★ Elite",IF(I8&gt;=21,"Strong",IF(I8&gt;=15,"Fair","Weak"))))</f>
-        <v>★ Elite</v>
+        <v>Strong</v>
+      </c>
+      <c r="K8" s="12" t="n">
+        <f aca="false">IF(I8="",0,I8)</f>
+        <v>26</v>
       </c>
       <c r="M8" s="12" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1883,13 +1926,13 @@
         <v>5</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E9" s="9" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>9</v>
@@ -1898,15 +1941,22 @@
         <v>9</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I9" s="11" t="n">
         <f aca="false">IF(COUNT(F9:H9)=0,"",SUM(F9:H9))</f>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="J9" s="11" t="str">
         <f aca="false">IF(I9="","",IF(I9&gt;=27,"★ Elite",IF(I9&gt;=21,"Strong",IF(I9&gt;=15,"Fair","Weak"))))</f>
-        <v>★ Elite</v>
+        <v>Strong</v>
+      </c>
+      <c r="K9" s="12" t="n">
+        <f aca="false">IF(I9="",0,I9)</f>
+        <v>26</v>
+      </c>
+      <c r="M9" s="12" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1914,22 +1964,22 @@
         <v>6</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G10" s="10" t="n">
         <v>9</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I10" s="11" t="n">
         <f aca="false">IF(COUNT(F10:H10)=0,"",SUM(F10:H10))</f>
@@ -1939,36 +1989,50 @@
         <f aca="false">IF(I10="","",IF(I10&gt;=27,"★ Elite",IF(I10&gt;=21,"Strong",IF(I10&gt;=15,"Fair","Weak"))))</f>
         <v>Strong</v>
       </c>
+      <c r="K10" s="12" t="n">
+        <f aca="false">IF(I10="",0,I10)</f>
+        <v>26</v>
+      </c>
+      <c r="M10" s="12" t="s">
+        <v>34</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="8" t="n">
         <v>7</v>
       </c>
       <c r="C11" s="9" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="E11" s="9" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G11" s="10" t="n">
         <v>9</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I11" s="11" t="n">
         <f aca="false">IF(COUNT(F11:H11)=0,"",SUM(F11:H11))</f>
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="J11" s="11" t="str">
         <f aca="false">IF(I11="","",IF(I11&gt;=27,"★ Elite",IF(I11&gt;=21,"Strong",IF(I11&gt;=15,"Fair","Weak"))))</f>
-        <v>★ Elite</v>
+        <v>Strong</v>
+      </c>
+      <c r="K11" s="12" t="n">
+        <f aca="false">IF(I11="",0,I11)</f>
+        <v>25</v>
+      </c>
+      <c r="M11" s="12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1976,13 +2040,13 @@
         <v>8</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F12" s="10" t="n">
         <v>8</v>
@@ -2001,28 +2065,32 @@
         <f aca="false">IF(I12="","",IF(I12&gt;=27,"★ Elite",IF(I12&gt;=21,"Strong",IF(I12&gt;=15,"Fair","Weak"))))</f>
         <v>Strong</v>
       </c>
+      <c r="K12" s="12" t="n">
+        <f aca="false">IF(I12="",0,I12)</f>
+        <v>25</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="8" t="n">
         <v>9</v>
       </c>
       <c r="C13" s="9" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G13" s="10" t="n">
         <v>8</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I13" s="11" t="n">
         <f aca="false">IF(COUNT(F13:H13)=0,"",SUM(F13:H13))</f>
@@ -2032,62 +2100,114 @@
         <f aca="false">IF(I13="","",IF(I13&gt;=27,"★ Elite",IF(I13&gt;=21,"Strong",IF(I13&gt;=15,"Fair","Weak"))))</f>
         <v>Strong</v>
       </c>
+      <c r="K13" s="12" t="n">
+        <f aca="false">IF(I13="",0,I13)</f>
+        <v>25</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="8" t="n">
         <v>10</v>
       </c>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="11" t="str">
+      <c r="C14" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="I14" s="11" t="n">
         <f aca="false">IF(COUNT(F14:H14)=0,"",SUM(F14:H14))</f>
-        <v/>
+        <v>24</v>
       </c>
       <c r="J14" s="11" t="str">
         <f aca="false">IF(I14="","",IF(I14&gt;=27,"★ Elite",IF(I14&gt;=21,"Strong",IF(I14&gt;=15,"Fair","Weak"))))</f>
-        <v/>
+        <v>Strong</v>
+      </c>
+      <c r="K14" s="12" t="n">
+        <f aca="false">IF(I14="",0,I14)</f>
+        <v>24</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="n">
         <v>11</v>
       </c>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="11" t="str">
+      <c r="C15" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="I15" s="11" t="n">
         <f aca="false">IF(COUNT(F15:H15)=0,"",SUM(F15:H15))</f>
-        <v/>
+        <v>20</v>
       </c>
       <c r="J15" s="11" t="str">
         <f aca="false">IF(I15="","",IF(I15&gt;=27,"★ Elite",IF(I15&gt;=21,"Strong",IF(I15&gt;=15,"Fair","Weak"))))</f>
-        <v/>
+        <v>Fair</v>
+      </c>
+      <c r="K15" s="12" t="n">
+        <f aca="false">IF(I15="",0,I15)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="8" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="11" t="str">
+      <c r="C16" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I16" s="11" t="n">
         <f aca="false">IF(COUNT(F16:H16)=0,"",SUM(F16:H16))</f>
-        <v/>
+        <v>23</v>
       </c>
       <c r="J16" s="11" t="str">
         <f aca="false">IF(I16="","",IF(I16&gt;=27,"★ Elite",IF(I16&gt;=21,"Strong",IF(I16&gt;=15,"Fair","Weak"))))</f>
-        <v/>
+        <v>Strong</v>
+      </c>
+      <c r="K16" s="12" t="n">
+        <f aca="false">IF(I16="",0,I16)</f>
+        <v>23</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2108,6 +2228,10 @@
         <f aca="false">IF(I17="","",IF(I17&gt;=27,"★ Elite",IF(I17&gt;=21,"Strong",IF(I17&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K17" s="12" t="n">
+        <f aca="false">IF(I17="",0,I17)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="n">
@@ -2127,6 +2251,10 @@
         <f aca="false">IF(I18="","",IF(I18&gt;=27,"★ Elite",IF(I18&gt;=21,"Strong",IF(I18&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K18" s="12" t="n">
+        <f aca="false">IF(I18="",0,I18)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="8" t="n">
@@ -2146,6 +2274,10 @@
         <f aca="false">IF(I19="","",IF(I19&gt;=27,"★ Elite",IF(I19&gt;=21,"Strong",IF(I19&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K19" s="12" t="n">
+        <f aca="false">IF(I19="",0,I19)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="8" t="n">
@@ -2165,6 +2297,10 @@
         <f aca="false">IF(I20="","",IF(I20&gt;=27,"★ Elite",IF(I20&gt;=21,"Strong",IF(I20&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K20" s="12" t="n">
+        <f aca="false">IF(I20="",0,I20)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="8" t="n">
@@ -2184,6 +2320,10 @@
         <f aca="false">IF(I21="","",IF(I21&gt;=27,"★ Elite",IF(I21&gt;=21,"Strong",IF(I21&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K21" s="12" t="n">
+        <f aca="false">IF(I21="",0,I21)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="8" t="n">
@@ -2203,6 +2343,10 @@
         <f aca="false">IF(I22="","",IF(I22&gt;=27,"★ Elite",IF(I22&gt;=21,"Strong",IF(I22&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K22" s="12" t="n">
+        <f aca="false">IF(I22="",0,I22)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="8" t="n">
@@ -2222,6 +2366,10 @@
         <f aca="false">IF(I23="","",IF(I23&gt;=27,"★ Elite",IF(I23&gt;=21,"Strong",IF(I23&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K23" s="12" t="n">
+        <f aca="false">IF(I23="",0,I23)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="8" t="n">
@@ -2241,6 +2389,10 @@
         <f aca="false">IF(I24="","",IF(I24&gt;=27,"★ Elite",IF(I24&gt;=21,"Strong",IF(I24&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K24" s="12" t="n">
+        <f aca="false">IF(I24="",0,I24)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="8" t="n">
@@ -2260,6 +2412,10 @@
         <f aca="false">IF(I25="","",IF(I25&gt;=27,"★ Elite",IF(I25&gt;=21,"Strong",IF(I25&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K25" s="12" t="n">
+        <f aca="false">IF(I25="",0,I25)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="8" t="n">
@@ -2279,6 +2435,10 @@
         <f aca="false">IF(I26="","",IF(I26&gt;=27,"★ Elite",IF(I26&gt;=21,"Strong",IF(I26&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K26" s="12" t="n">
+        <f aca="false">IF(I26="",0,I26)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="8" t="n">
@@ -2298,6 +2458,10 @@
         <f aca="false">IF(I27="","",IF(I27&gt;=27,"★ Elite",IF(I27&gt;=21,"Strong",IF(I27&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K27" s="12" t="n">
+        <f aca="false">IF(I27="",0,I27)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="8" t="n">
@@ -2317,6 +2481,10 @@
         <f aca="false">IF(I28="","",IF(I28&gt;=27,"★ Elite",IF(I28&gt;=21,"Strong",IF(I28&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K28" s="12" t="n">
+        <f aca="false">IF(I28="",0,I28)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="8" t="n">
@@ -2336,6 +2504,10 @@
         <f aca="false">IF(I29="","",IF(I29&gt;=27,"★ Elite",IF(I29&gt;=21,"Strong",IF(I29&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K29" s="12" t="n">
+        <f aca="false">IF(I29="",0,I29)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="8" t="n">
@@ -2355,6 +2527,10 @@
         <f aca="false">IF(I30="","",IF(I30&gt;=27,"★ Elite",IF(I30&gt;=21,"Strong",IF(I30&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K30" s="12" t="n">
+        <f aca="false">IF(I30="",0,I30)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="8" t="n">
@@ -2374,6 +2550,10 @@
         <f aca="false">IF(I31="","",IF(I31&gt;=27,"★ Elite",IF(I31&gt;=21,"Strong",IF(I31&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K31" s="12" t="n">
+        <f aca="false">IF(I31="",0,I31)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="8" t="n">
@@ -2393,6 +2573,10 @@
         <f aca="false">IF(I32="","",IF(I32&gt;=27,"★ Elite",IF(I32&gt;=21,"Strong",IF(I32&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K32" s="12" t="n">
+        <f aca="false">IF(I32="",0,I32)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="8" t="n">
@@ -2412,6 +2596,10 @@
         <f aca="false">IF(I33="","",IF(I33&gt;=27,"★ Elite",IF(I33&gt;=21,"Strong",IF(I33&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K33" s="12" t="n">
+        <f aca="false">IF(I33="",0,I33)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="8" t="n">
@@ -2431,6 +2619,10 @@
         <f aca="false">IF(I34="","",IF(I34&gt;=27,"★ Elite",IF(I34&gt;=21,"Strong",IF(I34&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K34" s="12" t="n">
+        <f aca="false">IF(I34="",0,I34)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="8" t="n">
@@ -2450,6 +2642,10 @@
         <f aca="false">IF(I35="","",IF(I35&gt;=27,"★ Elite",IF(I35&gt;=21,"Strong",IF(I35&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K35" s="12" t="n">
+        <f aca="false">IF(I35="",0,I35)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="8" t="n">
@@ -2469,6 +2665,10 @@
         <f aca="false">IF(I36="","",IF(I36&gt;=27,"★ Elite",IF(I36&gt;=21,"Strong",IF(I36&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K36" s="12" t="n">
+        <f aca="false">IF(I36="",0,I36)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B37" s="8" t="n">
@@ -2488,6 +2688,10 @@
         <f aca="false">IF(I37="","",IF(I37&gt;=27,"★ Elite",IF(I37&gt;=21,"Strong",IF(I37&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K37" s="12" t="n">
+        <f aca="false">IF(I37="",0,I37)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="8" t="n">
@@ -2507,6 +2711,10 @@
         <f aca="false">IF(I38="","",IF(I38&gt;=27,"★ Elite",IF(I38&gt;=21,"Strong",IF(I38&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K38" s="12" t="n">
+        <f aca="false">IF(I38="",0,I38)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B39" s="8" t="n">
@@ -2526,6 +2734,10 @@
         <f aca="false">IF(I39="","",IF(I39&gt;=27,"★ Elite",IF(I39&gt;=21,"Strong",IF(I39&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K39" s="12" t="n">
+        <f aca="false">IF(I39="",0,I39)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="8" t="n">
@@ -2545,6 +2757,10 @@
         <f aca="false">IF(I40="","",IF(I40&gt;=27,"★ Elite",IF(I40&gt;=21,"Strong",IF(I40&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K40" s="12" t="n">
+        <f aca="false">IF(I40="",0,I40)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="8" t="n">
@@ -2564,6 +2780,10 @@
         <f aca="false">IF(I41="","",IF(I41&gt;=27,"★ Elite",IF(I41&gt;=21,"Strong",IF(I41&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K41" s="12" t="n">
+        <f aca="false">IF(I41="",0,I41)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="8" t="n">
@@ -2583,6 +2803,10 @@
         <f aca="false">IF(I42="","",IF(I42&gt;=27,"★ Elite",IF(I42&gt;=21,"Strong",IF(I42&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K42" s="12" t="n">
+        <f aca="false">IF(I42="",0,I42)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="8" t="n">
@@ -2602,6 +2826,10 @@
         <f aca="false">IF(I43="","",IF(I43&gt;=27,"★ Elite",IF(I43&gt;=21,"Strong",IF(I43&gt;=15,"Fair","Weak"))))</f>
         <v/>
       </c>
+      <c r="K43" s="12" t="n">
+        <f aca="false">IF(I43="",0,I43)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="8" t="n">
@@ -2620,6 +2848,10 @@
       <c r="J44" s="11" t="str">
         <f aca="false">IF(I44="","",IF(I44&gt;=27,"★ Elite",IF(I44&gt;=21,"Strong",IF(I44&gt;=15,"Fair","Weak"))))</f>
         <v/>
+      </c>
+      <c r="K44" s="12" t="n">
+        <f aca="false">IF(I44="",0,I44)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2646,7 +2878,7 @@
       <formula2>10</formula2>
     </dataValidation>
     <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E5:E44" type="list">
-      <formula1>$M$5:$M$8</formula1>
+      <formula1>$M$5:$M$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -2666,28 +2898,24 @@
     <tabColor rgb="FF6AAA64"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:J7"/>
+  <dimension ref="B2:M7"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="20"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="5" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="8"/>
   </cols>
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="6" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>17</v>
@@ -2696,137 +2924,182 @@
         <v>18</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>42</v>
+        <v>46</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="L4" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="n">
-        <f aca="false">RANK(I5,$I$5:$I$7)</f>
-        <v>2</v>
+        <f aca="false">RANK(L5,$L$5:$L$7)</f>
+        <v>1</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Submissions!$D:$D,MATCH($C5,Submissions!$C:$C,0)),"")</f>
-        <v>Steward</v>
+        <v>Rob (human steward)</v>
       </c>
       <c r="E5" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C5,Submissions!$E:$E,"More Minds are better than one Mind: Research Quest")</f>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="Special Skills using X")*Submissions!$K$5:$K$44))</f>
+        <v>28</v>
+      </c>
+      <c r="F5" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="More Minds are better than one Mind: Research Quest")*Submissions!$K$5:$K$44))</f>
+        <v>28</v>
+      </c>
+      <c r="G5" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="Cross Word Puzzle")*Submissions!$K$5:$K$44))</f>
         <v>27</v>
       </c>
-      <c r="F5" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C5,Submissions!$E:$E,"Mindsheets Masterpiece and Debugging")</f>
-        <v>0</v>
-      </c>
-      <c r="G5" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C5,Submissions!$E:$E,"Cross Word Puzzle")</f>
-        <v>28</v>
-      </c>
       <c r="H5" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C5,Submissions!$E:$E,"Calm before the Storm")</f>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="Calm before the Storm")*Submissions!$K$5:$K$44))</f>
         <v>26</v>
       </c>
-      <c r="I5" s="17" t="n">
-        <f aca="false">SUM(E5:H5)</f>
-        <v>81</v>
-      </c>
-      <c r="J5" s="15" t="str">
+      <c r="I5" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="AstroMesh: Minds &amp; MCP Mashup Challenge")*Submissions!$K$5:$K$44))</f>
+        <v>26</v>
+      </c>
+      <c r="J5" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="Minds Building Chatbots Challenge")*Submissions!$K$5:$K$44))</f>
+        <v>26</v>
+      </c>
+      <c r="K5" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C5)*(Submissions!$E$5:$E$44="Mindsheets Masterpiece and Debugging")*Submissions!$K$5:$K$44))</f>
+        <v>25</v>
+      </c>
+      <c r="L5" s="17" t="n">
+        <f aca="false">SUM(E5:K5)</f>
+        <v>186</v>
+      </c>
+      <c r="M5" s="15" t="str">
         <f aca="false">IF(B5=1,"🥇",IF(B5=2,"🥈",IF(B5=3,"🥉","")))</f>
-        <v>🥈</v>
+        <v>🥇</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13" t="n">
-        <f aca="false">RANK(I6,$I$5:$I$7)</f>
-        <v>1</v>
+        <f aca="false">RANK(L6,$L$5:$L$7)</f>
+        <v>2</v>
       </c>
       <c r="C6" s="18" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="D6" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Submissions!$D:$D,MATCH($C6,Submissions!$C:$C,0)),"")</f>
-        <v>nip0r</v>
+        <v>(fictional)</v>
       </c>
       <c r="E6" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C6,Submissions!$E:$E,"More Minds are better than one Mind: Research Quest")</f>
-        <v>28</v>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="Special Skills using X")*Submissions!$K$5:$K$44))</f>
+        <v>25</v>
       </c>
       <c r="F6" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C6,Submissions!$E:$E,"Mindsheets Masterpiece and Debugging")</f>
-        <v>27</v>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="More Minds are better than one Mind: Research Quest")*Submissions!$K$5:$K$44))</f>
+        <v>25</v>
       </c>
       <c r="G6" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C6,Submissions!$E:$E,"Cross Word Puzzle")</f>
-        <v>26</v>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="Cross Word Puzzle")*Submissions!$K$5:$K$44))</f>
+        <v>24</v>
       </c>
       <c r="H6" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C6,Submissions!$E:$E,"Calm before the Storm")</f>
-        <v>27</v>
-      </c>
-      <c r="I6" s="17" t="n">
-        <f aca="false">SUM(E6:H6)</f>
-        <v>108</v>
-      </c>
-      <c r="J6" s="15" t="str">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="Calm before the Storm")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
+      </c>
+      <c r="I6" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="AstroMesh: Minds &amp; MCP Mashup Challenge")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="Minds Building Chatbots Challenge")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
+      </c>
+      <c r="K6" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C6)*(Submissions!$E$5:$E$44="Mindsheets Masterpiece and Debugging")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
+      </c>
+      <c r="L6" s="17" t="n">
+        <f aca="false">SUM(E6:K6)</f>
+        <v>74</v>
+      </c>
+      <c r="M6" s="15" t="str">
         <f aca="false">IF(B6=1,"🥇",IF(B6=2,"🥈",IF(B6=3,"🥉","")))</f>
-        <v>🥇</v>
+        <v>🥈</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="n">
-        <f aca="false">RANK(I7,$I$5:$I$7)</f>
+        <f aca="false">RANK(L7,$L$5:$L$7)</f>
         <v>3</v>
       </c>
       <c r="C7" s="18" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="D7" s="15" t="str">
         <f aca="false">IFERROR(INDEX(Submissions!$D:$D,MATCH($C7,Submissions!$C:$C,0)),"")</f>
-        <v>Michael</v>
+        <v>(fictional)</v>
       </c>
       <c r="E7" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C7,Submissions!$E:$E,"More Minds are better than one Mind: Research Quest")</f>
-        <v>25</v>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="Special Skills using X")*Submissions!$K$5:$K$44))</f>
+        <v>20</v>
       </c>
       <c r="F7" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C7,Submissions!$E:$E,"Mindsheets Masterpiece and Debugging")</f>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="More Minds are better than one Mind: Research Quest")*Submissions!$K$5:$K$44))</f>
         <v>0</v>
       </c>
       <c r="G7" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C7,Submissions!$E:$E,"Cross Word Puzzle")</f>
-        <v>25</v>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="Cross Word Puzzle")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
       </c>
       <c r="H7" s="16" t="n">
-        <f aca="false">SUMIFS(Submissions!$I:$I,Submissions!$C:$C,$C7,Submissions!$E:$E,"Calm before the Storm")</f>
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="Calm before the Storm")*Submissions!$K$5:$K$44))</f>
+        <v>23</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="AstroMesh: Minds &amp; MCP Mashup Challenge")*Submissions!$K$5:$K$44))</f>
         <v>0</v>
       </c>
-      <c r="I7" s="17" t="n">
-        <f aca="false">SUM(E7:H7)</f>
-        <v>50</v>
-      </c>
-      <c r="J7" s="15" t="str">
+      <c r="J7" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="Minds Building Chatbots Challenge")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="16" t="n">
+        <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="Mindsheets Masterpiece and Debugging")*Submissions!$K$5:$K$44))</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="17" t="n">
+        <f aca="false">SUM(E7:K7)</f>
+        <v>43</v>
+      </c>
+      <c r="M7" s="15" t="str">
         <f aca="false">IF(B7=1,"🥇",IF(B7=2,"🥈",IF(B7=3,"🥉","")))</f>
         <v>🥉</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="I5:I7">
+  <conditionalFormatting sqref="L5:L7">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min" val="0"/>
@@ -2836,7 +3109,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:J7">
+  <conditionalFormatting sqref="B5:M7">
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
       <formula>$B5=1</formula>
     </cfRule>
@@ -2865,32 +3138,32 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>45</v>
+        <v>52</v>
       </c>
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
       <c r="E5" s="19" t="s">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="F5" s="19"/>
       <c r="G5" s="19"/>
       <c r="H5" s="19" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="I5" s="19"/>
       <c r="J5" s="19"/>
       <c r="K5" s="19" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="L5" s="19"/>
       <c r="M5" s="19"/>
@@ -2898,25 +3171,25 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="20" t="str">
         <f aca="false">INDEX(Leaderboard!C:C,MATCH(1,Leaderboard!B:B,0))</f>
-        <v>Minty</v>
+        <v>NeoBerlin</v>
       </c>
       <c r="C6" s="20"/>
       <c r="D6" s="20"/>
       <c r="E6" s="20" t="n">
-        <f aca="false">MAX(Leaderboard!I:I)</f>
-        <v>108</v>
+        <f aca="false">MAX(Leaderboard!L:L)</f>
+        <v>186</v>
       </c>
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
       <c r="H6" s="20" t="n">
-        <f aca="false">INDEX(Leaderboard!I:I,MATCH("NeoBerlin",Leaderboard!C:C,0))</f>
-        <v>81</v>
+        <f aca="false">INDEX(Leaderboard!L:L,MATCH("NeoBerlin",Leaderboard!C:C,0))</f>
+        <v>186</v>
       </c>
       <c r="I6" s="20"/>
       <c r="J6" s="20"/>
       <c r="K6" s="20" t="n">
-        <f aca="false">MAX(Leaderboard!I:I)-INDEX(Leaderboard!I:I,MATCH("NeoBerlin",Leaderboard!C:C,0))</f>
-        <v>27</v>
+        <f aca="false">MAX(Leaderboard!L:L)-INDEX(Leaderboard!L:L,MATCH("NeoBerlin",Leaderboard!C:C,0))</f>
+        <v>0</v>
       </c>
       <c r="L6" s="20"/>
       <c r="M6" s="20"/>
@@ -2937,7 +3210,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="21" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2945,7 +3218,7 @@
         <v>17</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>50</v>
+        <v>57</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2954,28 +3227,28 @@
         <v>NeoBerlin</v>
       </c>
       <c r="C12" s="15" t="n">
-        <f aca="false">Leaderboard!I5</f>
-        <v>81</v>
+        <f aca="false">Leaderboard!L5</f>
+        <v>186</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="22" t="str">
         <f aca="false">Leaderboard!C6</f>
-        <v>Minty</v>
+        <v>Demo-Alpha</v>
       </c>
       <c r="C13" s="15" t="n">
-        <f aca="false">Leaderboard!I6</f>
-        <v>108</v>
+        <f aca="false">Leaderboard!L6</f>
+        <v>74</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="22" t="str">
         <f aca="false">Leaderboard!C7</f>
-        <v>VARgentina</v>
+        <v>Demo-Beta</v>
       </c>
       <c r="C14" s="15" t="n">
-        <f aca="false">Leaderboard!I7</f>
-        <v>50</v>
+        <f aca="false">Leaderboard!L7</f>
+        <v>43</v>
       </c>
     </row>
   </sheetData>
@@ -3019,23 +3292,23 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="23" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>3</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>54</v>
+        <v>61</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3043,96 +3316,96 @@
         <v>18</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="22" t="s">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="C8" s="25" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="15" t="n">
-        <f aca="false">Leaderboard!I5</f>
-        <v>81</v>
+        <f aca="false">Leaderboard!L5</f>
+        <v>186</v>
       </c>
       <c r="E8" s="26" t="n">
         <f aca="false">SQRT(D8)</f>
-        <v>9</v>
+        <v>13.6381816969859</v>
       </c>
       <c r="F8" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E8/SUM($E$8:$E$11))</f>
-        <v>0.286968271990825</v>
+        <v>0.404730749394807</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">$D$5*F8</f>
-        <v>0.860904815972475</v>
+        <v>1.21419224818442</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="22" t="s">
-        <v>32</v>
+        <v>67</v>
       </c>
       <c r="C9" s="25" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="15" t="n">
-        <f aca="false">Leaderboard!I6</f>
-        <v>108</v>
+        <f aca="false">Leaderboard!L6</f>
+        <v>74</v>
       </c>
       <c r="E9" s="26" t="n">
         <f aca="false">SQRT(D9)</f>
-        <v>10.3923048454133</v>
+        <v>8.60232526704263</v>
       </c>
       <c r="F9" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E9/SUM($E$8:$E$11))</f>
-        <v>0.331362418165569</v>
+        <v>0.255285171383038</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">$D$5*F9</f>
-        <v>0.994087254496707</v>
+        <v>0.765855514149114</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="22" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="C10" s="25" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="15" t="n">
-        <f aca="false">Leaderboard!I7</f>
-        <v>50</v>
+        <f aca="false">Leaderboard!L7</f>
+        <v>43</v>
       </c>
       <c r="E10" s="26" t="n">
         <f aca="false">SQRT(D10)</f>
-        <v>7.07106781186548</v>
+        <v>6.557438524302</v>
       </c>
       <c r="F10" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E10/SUM($E$8:$E$11))</f>
-        <v>0.225463567900109</v>
+        <v>0.194600502253001</v>
       </c>
       <c r="G10" s="28" t="n">
         <f aca="false">$D$5*F10</f>
-        <v>0.676390703700326</v>
+        <v>0.583801506759001</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="22" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C11" s="25" t="n">
         <v>12</v>
@@ -3147,16 +3420,16 @@
       </c>
       <c r="F11" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E11/SUM($E$8:$E$11))</f>
-        <v>0.156205741943497</v>
+        <v>0.145383576969155</v>
       </c>
       <c r="G11" s="28" t="n">
         <f aca="false">$D$5*F11</f>
-        <v>0.468617225830492</v>
+        <v>0.436150730907464</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="29" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="C12" s="30"/>
       <c r="D12" s="30"/>
@@ -3172,17 +3445,17 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="2" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="2" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -3225,12 +3498,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>65</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3238,19 +3511,19 @@
         <v>16</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>67</v>
+        <v>76</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3258,19 +3531,19 @@
         <v>1</v>
       </c>
       <c r="C6" s="34" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="D6" s="34" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
       <c r="E6" s="34" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3278,19 +3551,19 @@
         <v>2</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="D7" s="34" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="E7" s="34" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3298,19 +3571,19 @@
         <v>3</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
       <c r="E8" s="34" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>85</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3318,19 +3591,19 @@
         <v>4</v>
       </c>
       <c r="C9" s="34" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="D9" s="34" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
       <c r="E9" s="34" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="F9" s="9" t="s">
-        <v>89</v>
+        <v>98</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3338,24 +3611,24 @@
         <v>5</v>
       </c>
       <c r="C10" s="34" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D10" s="34" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="E10" s="34" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="35" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -3392,12 +3665,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3405,62 +3678,62 @@
         <v>19</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
-        <v>108</v>
+        <v>29</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>28</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>26.5</v>
+        <v>27.5</v>
       </c>
       <c r="G6" s="10" t="n">
-        <v>1.52</v>
+        <v>0.71</v>
       </c>
       <c r="H6" s="36" t="n">
         <f aca="false">IF($E6&lt;2,"n/a",1-NORMDIST($C6,$F6,$G6,TRUE()))</f>
-        <v>0.161860024867321</v>
+        <v>0.240646222600921</v>
       </c>
       <c r="I6" s="37" t="n">
         <f aca="false">IF($E6&lt;2,"insufficient history",$C6*NORMDIST($C6,$F6,$G6,TRUE())+$F6*(1-NORMDIST($C6,$F6,$G6,TRUE()))+$G6*$G6*NORMDIST($C6,$F6,$G6,FALSE())-$C6)</f>
-        <v>0.129844598264178</v>
+        <v>0.100720443700393</v>
       </c>
       <c r="J6" s="38" t="str">
         <f aca="false">IF($E6&lt;2,"need &gt;=2 scores",IF($D6=0,"no attempts left",IF($I6&gt;=0.5,"SHOOT — best use of an attempt",IF($I6&gt;=0.15,"worthwhile","low return"))))</f>
@@ -3468,159 +3741,159 @@
       </c>
       <c r="K6" s="39" t="n">
         <f aca="false">IF(AND($D6&gt;0,$E6&gt;=2),$I6,-999)</f>
-        <v>0.129844598264178</v>
+        <v>0.100720443700393</v>
       </c>
       <c r="L6" s="40" t="str">
         <f aca="false">IF($E6&lt;2,"",REPT("|",ROUND(MAX($I6,0)*20,0)))</f>
-        <v>|||</v>
+        <v>||</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="34" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="33" t="n">
         <v>5</v>
       </c>
       <c r="F7" s="10" t="n">
-        <v>23.5</v>
+        <v>26.5</v>
       </c>
       <c r="G7" s="10" t="n">
-        <v>4.04</v>
+        <v>1.36</v>
       </c>
       <c r="H7" s="36" t="n">
         <f aca="false">IF($E7&lt;2,"n/a",1-NORMDIST($C7,$F7,$G7,TRUE()))</f>
-        <v>0.355211841857091</v>
+        <v>0.135026355547818</v>
       </c>
       <c r="I7" s="37" t="n">
         <f aca="false">IF($E7&lt;2,"insufficient history",$C7*NORMDIST($C7,$F7,$G7,TRUE())+$F7*(1-NORMDIST($C7,$F7,$G7,TRUE()))+$G7*$G7*NORMDIST($C7,$F7,$G7,FALSE())-$C7)</f>
-        <v>0.971559588914271</v>
+        <v>0.0927811494462922</v>
       </c>
       <c r="J7" s="38" t="str">
         <f aca="false">IF($E7&lt;2,"need &gt;=2 scores",IF($D7=0,"no attempts left",IF($I7&gt;=0.5,"SHOOT — best use of an attempt",IF($I7&gt;=0.15,"worthwhile","low return"))))</f>
-        <v>SHOOT — best use of an attempt</v>
+        <v>low return</v>
       </c>
       <c r="K7" s="39" t="n">
         <f aca="false">IF(AND($D7&gt;0,$E7&gt;=2),$I7,-999)</f>
-        <v>0.971559588914271</v>
+        <v>0.0927811494462922</v>
       </c>
       <c r="L7" s="40" t="str">
         <f aca="false">IF($E7&lt;2,"",REPT("|",ROUND(MAX($I7,0)*20,0)))</f>
-        <v>|||||||||||||||||||</v>
+        <v>||</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="34" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="F8" s="10" t="n">
         <v>25</v>
       </c>
-      <c r="D8" s="10" t="n">
-        <v>2</v>
-      </c>
-      <c r="E8" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>23.5</v>
-      </c>
       <c r="G8" s="10" t="n">
-        <v>1.67</v>
+        <v>2.23</v>
       </c>
       <c r="H8" s="36" t="n">
         <f aca="false">IF($E8&lt;2,"n/a",1-NORMDIST($C8,$F8,$G8,TRUE()))</f>
-        <v>0.184538509157721</v>
+        <v>0.184896550093709</v>
       </c>
       <c r="I8" s="37" t="n">
         <f aca="false">IF($E8&lt;2,"insufficient history",$C8*NORMDIST($C8,$F8,$G8,TRUE())+$F8*(1-NORMDIST($C8,$F8,$G8,TRUE()))+$G8*$G8*NORMDIST($C8,$F8,$G8,FALSE())-$C8)</f>
-        <v>0.168272896693331</v>
+        <v>0.225252782691307</v>
       </c>
       <c r="J8" s="38" t="str">
         <f aca="false">IF($E8&lt;2,"need &gt;=2 scores",IF($D8=0,"no attempts left",IF($I8&gt;=0.5,"SHOOT — best use of an attempt",IF($I8&gt;=0.15,"worthwhile","low return"))))</f>
-        <v>worthwhile</v>
+        <v>no attempts left</v>
       </c>
       <c r="K8" s="39" t="n">
         <f aca="false">IF(AND($D8&gt;0,$E8&gt;=2),$I8,-999)</f>
-        <v>0.168272896693331</v>
+        <v>-999</v>
       </c>
       <c r="L8" s="40" t="str">
         <f aca="false">IF($E8&lt;2,"",REPT("|",ROUND(MAX($I8,0)*20,0)))</f>
-        <v>|||</v>
+        <v>|||||</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="34" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F9" s="10" t="n">
-        <v>22.5</v>
+        <v>24.5</v>
       </c>
       <c r="G9" s="10" t="n">
-        <v>1.72</v>
+        <v>1.76</v>
       </c>
       <c r="H9" s="36" t="n">
         <f aca="false">IF($E9&lt;2,"n/a",1-NORMDIST($C9,$F9,$G9,TRUE()))</f>
-        <v>0.0730441029274296</v>
+        <v>0.197031369686655</v>
       </c>
       <c r="I9" s="37" t="n">
         <f aca="false">IF($E9&lt;2,"insufficient history",$C9*NORMDIST($C9,$F9,$G9,TRUE())+$F9*(1-NORMDIST($C9,$F9,$G9,TRUE()))+$G9*$G9*NORMDIST($C9,$F9,$G9,FALSE())-$C9)</f>
-        <v>0.0559988819604165</v>
+        <v>0.192760847660367</v>
       </c>
       <c r="J9" s="38" t="str">
         <f aca="false">IF($E9&lt;2,"need &gt;=2 scores",IF($D9=0,"no attempts left",IF($I9&gt;=0.5,"SHOOT — best use of an attempt",IF($I9&gt;=0.15,"worthwhile","low return"))))</f>
-        <v>low return</v>
+        <v>worthwhile</v>
       </c>
       <c r="K9" s="39" t="n">
         <f aca="false">IF(AND($D9&gt;0,$E9&gt;=2),$I9,-999)</f>
-        <v>0.0559988819604165</v>
+        <v>0.192760847660367</v>
       </c>
       <c r="L9" s="40" t="str">
         <f aca="false">IF($E9&lt;2,"",REPT("|",ROUND(MAX($I9,0)*20,0)))</f>
-        <v>|</v>
+        <v>||||</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="34" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>26</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F10" s="10" t="n">
-        <v>23</v>
+        <v>23.5</v>
       </c>
       <c r="G10" s="10" t="n">
-        <v>1.9</v>
+        <v>1.17</v>
       </c>
       <c r="H10" s="36" t="n">
         <f aca="false">IF($E10&lt;2,"n/a",1-NORMDIST($C10,$F10,$G10,TRUE()))</f>
-        <v>0.0571740648711003</v>
+        <v>0.0163090784888628</v>
       </c>
       <c r="I10" s="37" t="n">
         <f aca="false">IF($E10&lt;2,"insufficient history",$C10*NORMDIST($C10,$F10,$G10,TRUE())+$F10*(1-NORMDIST($C10,$F10,$G10,TRUE()))+$G10*$G10*NORMDIST($C10,$F10,$G10,FALSE())-$C10)</f>
-        <v>0.0463989413775963</v>
+        <v>0.00683362959041389</v>
       </c>
       <c r="J10" s="38" t="str">
         <f aca="false">IF($E10&lt;2,"need &gt;=2 scores",IF($D10=0,"no attempts left",IF($I10&gt;=0.5,"SHOOT — best use of an attempt",IF($I10&gt;=0.15,"worthwhile","low return"))))</f>
@@ -3628,39 +3901,39 @@
       </c>
       <c r="K10" s="39" t="n">
         <f aca="false">IF(AND($D10&gt;0,$E10&gt;=2),$I10,-999)</f>
-        <v>0.0463989413775963</v>
+        <v>0.00683362959041389</v>
       </c>
       <c r="L10" s="40" t="str">
         <f aca="false">IF($E10&lt;2,"",REPT("|",ROUND(MAX($I10,0)*20,0)))</f>
-        <v>|</v>
+        <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="34" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>26</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E11" s="33" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="G11" s="10" t="n">
-        <v>1.3</v>
+        <v>1.76</v>
       </c>
       <c r="H11" s="36" t="n">
         <f aca="false">IF($E11&lt;2,"n/a",1-NORMDIST($C11,$F11,$G11,TRUE()))</f>
-        <v>0.0272351950137387</v>
+        <v>0.0441396158580674</v>
       </c>
       <c r="I11" s="37" t="n">
         <f aca="false">IF($E11&lt;2,"insufficient history",$C11*NORMDIST($C11,$F11,$G11,TRUE())+$F11*(1-NORMDIST($C11,$F11,$G11,TRUE()))+$G11*$G11*NORMDIST($C11,$F11,$G11,FALSE())-$C11)</f>
-        <v>0.0135315434974004</v>
+        <v>0.0318316934919807</v>
       </c>
       <c r="J11" s="38" t="str">
         <f aca="false">IF($E11&lt;2,"need &gt;=2 scores",IF($D11=0,"no attempts left",IF($I11&gt;=0.5,"SHOOT — best use of an attempt",IF($I11&gt;=0.15,"worthwhile","low return"))))</f>
@@ -3668,56 +3941,56 @@
       </c>
       <c r="K11" s="39" t="n">
         <f aca="false">IF(AND($D11&gt;0,$E11&gt;=2),$I11,-999)</f>
-        <v>0.0135315434974004</v>
+        <v>0.0318316934919807</v>
       </c>
       <c r="L11" s="40" t="str">
         <f aca="false">IF($E11&lt;2,"",REPT("|",ROUND(MAX($I11,0)*20,0)))</f>
-        <v/>
+        <v>|</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="34" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C12" s="10" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>26</v>
+        <v>22.5</v>
       </c>
       <c r="G12" s="10" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="H12" s="36" t="str">
+        <v>3.3</v>
+      </c>
+      <c r="H12" s="36" t="n">
         <f aca="false">IF($E12&lt;2,"n/a",1-NORMDIST($C12,$F12,$G12,TRUE()))</f>
-        <v>n/a</v>
-      </c>
-      <c r="I12" s="37" t="str">
+        <v>0.224352498756818</v>
+      </c>
+      <c r="I12" s="37" t="n">
         <f aca="false">IF($E12&lt;2,"insufficient history",$C12*NORMDIST($C12,$F12,$G12,TRUE())+$F12*(1-NORMDIST($C12,$F12,$G12,TRUE()))+$G12*$G12*NORMDIST($C12,$F12,$G12,FALSE())-$C12)</f>
-        <v>insufficient history</v>
+        <v>0.427213607902583</v>
       </c>
       <c r="J12" s="38" t="str">
         <f aca="false">IF($E12&lt;2,"need &gt;=2 scores",IF($D12=0,"no attempts left",IF($I12&gt;=0.5,"SHOOT — best use of an attempt",IF($I12&gt;=0.15,"worthwhile","low return"))))</f>
-        <v>need &gt;=2 scores</v>
+        <v>worthwhile</v>
       </c>
       <c r="K12" s="39" t="n">
         <f aca="false">IF(AND($D12&gt;0,$E12&gt;=2),$I12,-999)</f>
-        <v>-999</v>
+        <v>0.427213607902583</v>
       </c>
       <c r="L12" s="40" t="str">
         <f aca="false">IF($E12&lt;2,"",REPT("|",ROUND(MAX($I12,0)*20,0)))</f>
-        <v/>
+        <v>|||||||||</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="D14" s="41" t="str">
         <f aca="false">INDEX($B$6:$B$12,MATCH(MAX($K$6:$K$12),$K$6:$K$12,0))</f>
@@ -3726,7 +3999,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="42" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C15" s="42"/>
       <c r="D15" s="42"/>

</xml_diff>

<commit_message>
mindsheets: fix static Best column found by human steward; live from Leaderboard; more demo variation
</commit_message>
<xml_diff>
--- a/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
+++ b/mindsheets/BattleOfTheMinds_Scoreboard.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="129">
   <si>
     <t xml:space="preserve">BATTLE OF THE MINDS</t>
   </si>
@@ -271,82 +271,97 @@
     <t xml:space="preserve">Pass?</t>
   </si>
   <si>
-    <t xml:space="preserve">Recommendation excludes an event with no attempts left</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Next Best Move D7 (Mindsheets Left): 2 -&gt; 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D14 switches to 'Calm before the Storm'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calm before the Storm (Excel)</t>
+    <t xml:space="preserve">Cross-app check: Apple Numbers, first build</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open a build written without cached values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values shown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ALL CELLS BLANK - Numbers does not recalculate imported formulas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cross-app check: Apple Numbers, after fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Open build with fullCalcOnLoad + baked-in values</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values shown AND live recalculation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Values shown; recalculation only after editing the cell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PARTIAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Best-of-event: a WEAKER second submission must be ignored</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Submissions row 17: C=NeoBerlin, E=Mindsheets, F/G/H = 5/5/5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I17=15, J17='Fair'; Leaderboard K5 stays 25; L5 stays 186</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I17=15, Fair; K5=25; L5=186 (Excel, MacBook)</t>
   </si>
   <si>
     <t xml:space="preserve">Pass</t>
   </si>
   <si>
-    <t xml:space="preserve">EV reacts correctly to a lower spread</t>
-  </si>
-  <si>
-    <t xml:space="preserve">D7 back to 2; G7 (Mindsheets sigma): 4.04 -&gt; 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I7 drops 0.97 -&gt; ~0.03; verdict 'low return'; D14 -&gt; Calm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">as expected (Excel)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cross-app check: Apple Numbers, first build</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open build without cached values in Numbers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Values shown</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ALL CELLS BLANK - Numbers does not recalculate imported formulas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAIL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cross-app check: Apple Numbers, after fix</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Open build with fullCalcOnLoad + baked-in values</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Values shown AND live recalculation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Values shown; recalculation only after editing the cell</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PARTIAL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">New submission totals correctly</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Submissions F14=9; G14=8; H14=7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">I14 = 24; Grade = Strong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24; Strong</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Status: Ready — in Microsoft Excel and LibreOffice Calc, verified by the human steward. Apple Numbers displays every value but does not re-evaluate imported formulas until a cell is edited; that is a Numbers import behaviour, not a formula error, and it is listed above as test 3 (FAIL) and test 4 (PARTIAL) rather than omitted.</t>
+    <t xml:space="preserve">Best-of-event: a STRONGER second submission must take over</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same row: F/G/H = 10/10/9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I17=29, J17='Elite'; Leaderboard K5=29; L5=190; Dashboard H6=190</t>
+  </si>
+  <si>
+    <t xml:space="preserve">all as expected (Excel, MacBook)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Next Best Move reacts to a changed score</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After test 4 (Mindsheets best 25 -&gt; 29), read Next Best Move C12 and D14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C12 becomes 29, Mindsheets EV collapses, D14 -&gt; 'Calm before the Storm'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C12 STILL 25 and D14 still 'Mindsheets' - the tab never updated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same check after the fix (Best now read from the Leaderboard)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Repeat test 4, then read Next Best Move C12 / I12 / D14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C12 = 29; I12 falls 0.427 -&gt; 0.030; D14 -&gt; 'Calm before the Storm'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDING - awaiting the steward's re-test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PENDING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status: Partially Ready — tests 1-5 were run by the human steward in Excel on macOS; test 6 (the re-test of the fix he prompted) is still pending. Apple Numbers displays every value but does not re-evaluate imported formulas until a cell is edited; that is a Numbers import behaviour, not a formula error, and it is listed above as test 3 (FAIL) and test 4 (PARTIAL) rather than omitted.</t>
   </si>
   <si>
     <t xml:space="preserve">NEXT BEST MOVE  ·  where should the next attempt go?</t>
   </si>
   <si>
-    <t xml:space="preserve">Expected value of ONE more attempt, per event. Best/Left/n come straight from the tournament API (GET /api/compete/puzzles and /submissions/me) on 2026-07-28. Only light-blue cells are inputs. mu = average of the last two scores (steward's choice); sigma = spread of all scores so far.</t>
+    <t xml:space="preserve">Expected value of ONE more attempt, per event. Best/Left/n come straight from the tournament API (GET /api/compete/puzzles and /submissions/me) on 2026-07-28. Only light-blue cells are inputs; 'Best' is read live from the Leaderboard, so raising a score anywhere updates this tab and the recommendation. mu = average of the last two scores (steward's choice); sigma = spread of all scores so far.</t>
   </si>
   <si>
     <t xml:space="preserve">Best</t>
@@ -377,6 +392,9 @@
   </si>
   <si>
     <t xml:space="preserve">EV bar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">key</t>
   </si>
   <si>
     <t xml:space="preserve">More Minds are better than one</t>
@@ -651,7 +669,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -794,6 +812,10 @@
     </xf>
     <xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -1044,7 +1066,7 @@
                   <c:v>74</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>43</c:v>
+                  <c:v>65</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1052,11 +1074,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="50949338"/>
-        <c:axId val="45396134"/>
+        <c:axId val="88643215"/>
+        <c:axId val="15431527"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="50949338"/>
+        <c:axId val="88643215"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1089,7 +1111,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45396134"/>
+        <c:crossAx val="15431527"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1097,7 +1119,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="45396134"/>
+        <c:axId val="15431527"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1140,7 +1162,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="50949338"/>
+        <c:crossAx val="88643215"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2145,34 +2167,34 @@
         <v>11</v>
       </c>
       <c r="C15" s="9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D15" s="9" t="s">
         <v>37</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F15" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G15" s="10" t="n">
         <v>7</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I15" s="11" t="n">
         <f aca="false">IF(COUNT(F15:H15)=0,"",SUM(F15:H15))</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="J15" s="11" t="str">
         <f aca="false">IF(I15="","",IF(I15&gt;=27,"★ Elite",IF(I15&gt;=21,"Strong",IF(I15&gt;=15,"Fair","Weak"))))</f>
-        <v>Fair</v>
+        <v>Strong</v>
       </c>
       <c r="K15" s="12" t="n">
         <f aca="false">IF(I15="",0,I15)</f>
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2186,74 +2208,98 @@
         <v>37</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G16" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="I16" s="11" t="n">
         <f aca="false">IF(COUNT(F16:H16)=0,"",SUM(F16:H16))</f>
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="J16" s="11" t="str">
         <f aca="false">IF(I16="","",IF(I16&gt;=27,"★ Elite",IF(I16&gt;=21,"Strong",IF(I16&gt;=15,"Fair","Weak"))))</f>
-        <v>Strong</v>
+        <v>Fair</v>
       </c>
       <c r="K16" s="12" t="n">
         <f aca="false">IF(I16="",0,I16)</f>
-        <v>23</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="8" t="n">
         <v>13</v>
       </c>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="11" t="str">
+      <c r="C17" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G17" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H17" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I17" s="11" t="n">
         <f aca="false">IF(COUNT(F17:H17)=0,"",SUM(F17:H17))</f>
-        <v/>
+        <v>23</v>
       </c>
       <c r="J17" s="11" t="str">
         <f aca="false">IF(I17="","",IF(I17&gt;=27,"★ Elite",IF(I17&gt;=21,"Strong",IF(I17&gt;=15,"Fair","Weak"))))</f>
-        <v/>
+        <v>Strong</v>
       </c>
       <c r="K17" s="12" t="n">
         <f aca="false">IF(I17="",0,I17)</f>
-        <v>0</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="8" t="n">
         <v>14</v>
       </c>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="11" t="str">
+      <c r="C18" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="I18" s="11" t="n">
         <f aca="false">IF(COUNT(F18:H18)=0,"",SUM(F18:H18))</f>
-        <v/>
+        <v>22</v>
       </c>
       <c r="J18" s="11" t="str">
         <f aca="false">IF(I18="","",IF(I18&gt;=27,"★ Elite",IF(I18&gt;=21,"Strong",IF(I18&gt;=15,"Fair","Weak"))))</f>
-        <v/>
+        <v>Strong</v>
       </c>
       <c r="K18" s="12" t="n">
         <f aca="false">IF(I18="",0,I18)</f>
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3079,7 +3125,7 @@
       </c>
       <c r="I7" s="16" t="n">
         <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="AstroMesh: Minds &amp; MCP Mashup Challenge")*Submissions!$K$5:$K$44))</f>
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="J7" s="16" t="n">
         <f aca="false">SUMPRODUCT(MAX((Submissions!$C$5:$C$44=$C7)*(Submissions!$E$5:$E$44="Minds Building Chatbots Challenge")*Submissions!$K$5:$K$44))</f>
@@ -3091,7 +3137,7 @@
       </c>
       <c r="L7" s="17" t="n">
         <f aca="false">SUM(E7:K7)</f>
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="M7" s="15" t="str">
         <f aca="false">IF(B7=1,"🥇",IF(B7=2,"🥈",IF(B7=3,"🥉","")))</f>
@@ -3248,7 +3294,7 @@
       </c>
       <c r="C14" s="15" t="n">
         <f aca="false">Leaderboard!L7</f>
-        <v>43</v>
+        <v>65</v>
       </c>
     </row>
   </sheetData>
@@ -3348,11 +3394,11 @@
       </c>
       <c r="F8" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E8/SUM($E$8:$E$11))</f>
-        <v>0.404730749394807</v>
+        <v>0.387429146133106</v>
       </c>
       <c r="G8" s="28" t="n">
         <f aca="false">$D$5*F8</f>
-        <v>1.21419224818442</v>
+        <v>1.16228743839932</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3372,11 +3418,11 @@
       </c>
       <c r="F9" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E9/SUM($E$8:$E$11))</f>
-        <v>0.255285171383038</v>
+        <v>0.24437213163879</v>
       </c>
       <c r="G9" s="28" t="n">
         <f aca="false">$D$5*F9</f>
-        <v>0.765855514149114</v>
+        <v>0.733116394916371</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3388,19 +3434,19 @@
       </c>
       <c r="D10" s="15" t="n">
         <f aca="false">Leaderboard!L7</f>
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="E10" s="26" t="n">
         <f aca="false">SQRT(D10)</f>
-        <v>6.557438524302</v>
+        <v>8.06225774829855</v>
       </c>
       <c r="F10" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E10/SUM($E$8:$E$11))</f>
-        <v>0.194600502253001</v>
+        <v>0.22903006461768</v>
       </c>
       <c r="G10" s="28" t="n">
         <f aca="false">$D$5*F10</f>
-        <v>0.583801506759001</v>
+        <v>0.687090193853039</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3420,11 +3466,11 @@
       </c>
       <c r="F11" s="27" t="n">
         <f aca="false">IF(SUM($E$8:$E$11)=0,0,E11/SUM($E$8:$E$11))</f>
-        <v>0.145383576969155</v>
+        <v>0.139168657610424</v>
       </c>
       <c r="G11" s="28" t="n">
         <f aca="false">$D$5*F11</f>
-        <v>0.436150730907464</v>
+        <v>0.417505972831272</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3485,7 +3531,7 @@
     <tabColor rgb="FF6B7280"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:G12"/>
+  <dimension ref="B2:G13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="5"/>
@@ -3563,7 +3609,7 @@
         <v>89</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3571,19 +3617,19 @@
         <v>3</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D8" s="34" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E8" s="34" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3591,19 +3637,19 @@
         <v>4</v>
       </c>
       <c r="C9" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="D9" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="E9" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="G9" s="10" t="s">
         <v>95</v>
-      </c>
-      <c r="D9" s="34" t="s">
-        <v>96</v>
-      </c>
-      <c r="E9" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="F9" s="9" t="s">
-        <v>98</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3626,9 +3672,29 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B12" s="35" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B11" s="33" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="34" t="s">
         <v>104</v>
+      </c>
+      <c r="D11" s="34" t="s">
+        <v>105</v>
+      </c>
+      <c r="E11" s="34" t="s">
+        <v>106</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B13" s="35" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -3648,7 +3714,7 @@
     <tabColor rgb="FF6AAA64"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:L15"/>
+  <dimension ref="B2:N15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28"/>
@@ -3665,12 +3731,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3678,47 +3744,51 @@
         <v>19</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="L5" s="6" t="s">
-        <v>116</v>
+        <v>121</v>
+      </c>
+      <c r="N5" s="7" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N6,Leaderboard!$E$4:$K$4,0))</f>
         <v>28</v>
       </c>
       <c r="D6" s="10" t="n">
         <v>4</v>
       </c>
-      <c r="E6" s="33" t="n">
+      <c r="E6" s="10" t="n">
         <v>4</v>
       </c>
       <c r="F6" s="10" t="n">
@@ -3727,38 +3797,42 @@
       <c r="G6" s="10" t="n">
         <v>0.71</v>
       </c>
-      <c r="H6" s="36" t="n">
+      <c r="H6" s="37" t="n">
         <f aca="false">IF($E6&lt;2,"n/a",1-NORMDIST($C6,$F6,$G6,TRUE()))</f>
         <v>0.240646222600921</v>
       </c>
-      <c r="I6" s="37" t="n">
+      <c r="I6" s="38" t="n">
         <f aca="false">IF($E6&lt;2,"insufficient history",$C6*NORMDIST($C6,$F6,$G6,TRUE())+$F6*(1-NORMDIST($C6,$F6,$G6,TRUE()))+$G6*$G6*NORMDIST($C6,$F6,$G6,FALSE())-$C6)</f>
         <v>0.100720443700393</v>
       </c>
-      <c r="J6" s="38" t="str">
+      <c r="J6" s="39" t="str">
         <f aca="false">IF($E6&lt;2,"need &gt;=2 scores",IF($D6=0,"no attempts left",IF($I6&gt;=0.5,"SHOOT — best use of an attempt",IF($I6&gt;=0.15,"worthwhile","low return"))))</f>
         <v>low return</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="K6" s="40" t="n">
         <f aca="false">IF(AND($D6&gt;0,$E6&gt;=2),$I6,-999)</f>
         <v>0.100720443700393</v>
       </c>
-      <c r="L6" s="40" t="str">
+      <c r="L6" s="41" t="str">
         <f aca="false">IF($E6&lt;2,"",REPT("|",ROUND(MAX($I6,0)*20,0)))</f>
         <v>||</v>
       </c>
+      <c r="N6" s="12" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="34" t="s">
-        <v>117</v>
-      </c>
-      <c r="C7" s="10" t="n">
+        <v>123</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N7,Leaderboard!$E$4:$K$4,0))</f>
         <v>28</v>
       </c>
       <c r="D7" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="33" t="n">
+      <c r="E7" s="10" t="n">
         <v>5</v>
       </c>
       <c r="F7" s="10" t="n">
@@ -3767,38 +3841,42 @@
       <c r="G7" s="10" t="n">
         <v>1.36</v>
       </c>
-      <c r="H7" s="36" t="n">
+      <c r="H7" s="37" t="n">
         <f aca="false">IF($E7&lt;2,"n/a",1-NORMDIST($C7,$F7,$G7,TRUE()))</f>
         <v>0.135026355547818</v>
       </c>
-      <c r="I7" s="37" t="n">
+      <c r="I7" s="38" t="n">
         <f aca="false">IF($E7&lt;2,"insufficient history",$C7*NORMDIST($C7,$F7,$G7,TRUE())+$F7*(1-NORMDIST($C7,$F7,$G7,TRUE()))+$G7*$G7*NORMDIST($C7,$F7,$G7,FALSE())-$C7)</f>
         <v>0.0927811494462922</v>
       </c>
-      <c r="J7" s="38" t="str">
+      <c r="J7" s="39" t="str">
         <f aca="false">IF($E7&lt;2,"need &gt;=2 scores",IF($D7=0,"no attempts left",IF($I7&gt;=0.5,"SHOOT — best use of an attempt",IF($I7&gt;=0.15,"worthwhile","low return"))))</f>
         <v>low return</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="K7" s="40" t="n">
         <f aca="false">IF(AND($D7&gt;0,$E7&gt;=2),$I7,-999)</f>
         <v>0.0927811494462922</v>
       </c>
-      <c r="L7" s="40" t="str">
+      <c r="L7" s="41" t="str">
         <f aca="false">IF($E7&lt;2,"",REPT("|",ROUND(MAX($I7,0)*20,0)))</f>
         <v>||</v>
+      </c>
+      <c r="N7" s="12" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="34" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N8,Leaderboard!$E$4:$K$4,0))</f>
         <v>27</v>
       </c>
       <c r="D8" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="33" t="n">
+      <c r="E8" s="10" t="n">
         <v>7</v>
       </c>
       <c r="F8" s="10" t="n">
@@ -3807,38 +3885,42 @@
       <c r="G8" s="10" t="n">
         <v>2.23</v>
       </c>
-      <c r="H8" s="36" t="n">
+      <c r="H8" s="37" t="n">
         <f aca="false">IF($E8&lt;2,"n/a",1-NORMDIST($C8,$F8,$G8,TRUE()))</f>
         <v>0.184896550093709</v>
       </c>
-      <c r="I8" s="37" t="n">
+      <c r="I8" s="38" t="n">
         <f aca="false">IF($E8&lt;2,"insufficient history",$C8*NORMDIST($C8,$F8,$G8,TRUE())+$F8*(1-NORMDIST($C8,$F8,$G8,TRUE()))+$G8*$G8*NORMDIST($C8,$F8,$G8,FALSE())-$C8)</f>
         <v>0.225252782691307</v>
       </c>
-      <c r="J8" s="38" t="str">
+      <c r="J8" s="39" t="str">
         <f aca="false">IF($E8&lt;2,"need &gt;=2 scores",IF($D8=0,"no attempts left",IF($I8&gt;=0.5,"SHOOT — best use of an attempt",IF($I8&gt;=0.15,"worthwhile","low return"))))</f>
         <v>no attempts left</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="K8" s="40" t="n">
         <f aca="false">IF(AND($D8&gt;0,$E8&gt;=2),$I8,-999)</f>
         <v>-999</v>
       </c>
-      <c r="L8" s="40" t="str">
+      <c r="L8" s="41" t="str">
         <f aca="false">IF($E8&lt;2,"",REPT("|",ROUND(MAX($I8,0)*20,0)))</f>
         <v>|||||</v>
+      </c>
+      <c r="N8" s="12" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N9,Leaderboard!$E$4:$K$4,0))</f>
         <v>26</v>
       </c>
       <c r="D9" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="33" t="n">
+      <c r="E9" s="10" t="n">
         <v>7</v>
       </c>
       <c r="F9" s="10" t="n">
@@ -3847,38 +3929,42 @@
       <c r="G9" s="10" t="n">
         <v>1.76</v>
       </c>
-      <c r="H9" s="36" t="n">
+      <c r="H9" s="37" t="n">
         <f aca="false">IF($E9&lt;2,"n/a",1-NORMDIST($C9,$F9,$G9,TRUE()))</f>
         <v>0.197031369686655</v>
       </c>
-      <c r="I9" s="37" t="n">
+      <c r="I9" s="38" t="n">
         <f aca="false">IF($E9&lt;2,"insufficient history",$C9*NORMDIST($C9,$F9,$G9,TRUE())+$F9*(1-NORMDIST($C9,$F9,$G9,TRUE()))+$G9*$G9*NORMDIST($C9,$F9,$G9,FALSE())-$C9)</f>
         <v>0.192760847660367</v>
       </c>
-      <c r="J9" s="38" t="str">
+      <c r="J9" s="39" t="str">
         <f aca="false">IF($E9&lt;2,"need &gt;=2 scores",IF($D9=0,"no attempts left",IF($I9&gt;=0.5,"SHOOT — best use of an attempt",IF($I9&gt;=0.15,"worthwhile","low return"))))</f>
         <v>worthwhile</v>
       </c>
-      <c r="K9" s="39" t="n">
+      <c r="K9" s="40" t="n">
         <f aca="false">IF(AND($D9&gt;0,$E9&gt;=2),$I9,-999)</f>
         <v>0.192760847660367</v>
       </c>
-      <c r="L9" s="40" t="str">
+      <c r="L9" s="41" t="str">
         <f aca="false">IF($E9&lt;2,"",REPT("|",ROUND(MAX($I9,0)*20,0)))</f>
         <v>||||</v>
       </c>
+      <c r="N9" s="12" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="34" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="10" t="n">
+        <v>124</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N10,Leaderboard!$E$4:$K$4,0))</f>
         <v>26</v>
       </c>
       <c r="D10" s="10" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="33" t="n">
+      <c r="E10" s="10" t="n">
         <v>5</v>
       </c>
       <c r="F10" s="10" t="n">
@@ -3887,38 +3973,42 @@
       <c r="G10" s="10" t="n">
         <v>1.17</v>
       </c>
-      <c r="H10" s="36" t="n">
+      <c r="H10" s="37" t="n">
         <f aca="false">IF($E10&lt;2,"n/a",1-NORMDIST($C10,$F10,$G10,TRUE()))</f>
         <v>0.0163090784888628</v>
       </c>
-      <c r="I10" s="37" t="n">
+      <c r="I10" s="38" t="n">
         <f aca="false">IF($E10&lt;2,"insufficient history",$C10*NORMDIST($C10,$F10,$G10,TRUE())+$F10*(1-NORMDIST($C10,$F10,$G10,TRUE()))+$G10*$G10*NORMDIST($C10,$F10,$G10,FALSE())-$C10)</f>
         <v>0.00683362959041389</v>
       </c>
-      <c r="J10" s="38" t="str">
+      <c r="J10" s="39" t="str">
         <f aca="false">IF($E10&lt;2,"need &gt;=2 scores",IF($D10=0,"no attempts left",IF($I10&gt;=0.5,"SHOOT — best use of an attempt",IF($I10&gt;=0.15,"worthwhile","low return"))))</f>
         <v>low return</v>
       </c>
-      <c r="K10" s="39" t="n">
+      <c r="K10" s="40" t="n">
         <f aca="false">IF(AND($D10&gt;0,$E10&gt;=2),$I10,-999)</f>
         <v>0.00683362959041389</v>
       </c>
-      <c r="L10" s="40" t="str">
+      <c r="L10" s="41" t="str">
         <f aca="false">IF($E10&lt;2,"",REPT("|",ROUND(MAX($I10,0)*20,0)))</f>
         <v/>
+      </c>
+      <c r="N10" s="12" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="34" t="s">
-        <v>119</v>
-      </c>
-      <c r="C11" s="10" t="n">
+        <v>125</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N11,Leaderboard!$E$4:$K$4,0))</f>
         <v>26</v>
       </c>
       <c r="D11" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="33" t="n">
+      <c r="E11" s="10" t="n">
         <v>7</v>
       </c>
       <c r="F11" s="10" t="n">
@@ -3927,38 +4017,42 @@
       <c r="G11" s="10" t="n">
         <v>1.76</v>
       </c>
-      <c r="H11" s="36" t="n">
+      <c r="H11" s="37" t="n">
         <f aca="false">IF($E11&lt;2,"n/a",1-NORMDIST($C11,$F11,$G11,TRUE()))</f>
         <v>0.0441396158580674</v>
       </c>
-      <c r="I11" s="37" t="n">
+      <c r="I11" s="38" t="n">
         <f aca="false">IF($E11&lt;2,"insufficient history",$C11*NORMDIST($C11,$F11,$G11,TRUE())+$F11*(1-NORMDIST($C11,$F11,$G11,TRUE()))+$G11*$G11*NORMDIST($C11,$F11,$G11,FALSE())-$C11)</f>
         <v>0.0318316934919807</v>
       </c>
-      <c r="J11" s="38" t="str">
+      <c r="J11" s="39" t="str">
         <f aca="false">IF($E11&lt;2,"need &gt;=2 scores",IF($D11=0,"no attempts left",IF($I11&gt;=0.5,"SHOOT — best use of an attempt",IF($I11&gt;=0.15,"worthwhile","low return"))))</f>
         <v>low return</v>
       </c>
-      <c r="K11" s="39" t="n">
+      <c r="K11" s="40" t="n">
         <f aca="false">IF(AND($D11&gt;0,$E11&gt;=2),$I11,-999)</f>
         <v>0.0318316934919807</v>
       </c>
-      <c r="L11" s="40" t="str">
+      <c r="L11" s="41" t="str">
         <f aca="false">IF($E11&lt;2,"",REPT("|",ROUND(MAX($I11,0)*20,0)))</f>
         <v>|</v>
       </c>
+      <c r="N11" s="12" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="34" t="s">
-        <v>120</v>
-      </c>
-      <c r="C12" s="10" t="n">
+        <v>126</v>
+      </c>
+      <c r="C12" s="36" t="n">
+        <f aca="false">INDEX(Leaderboard!$E$5:$K$5,MATCH($N12,Leaderboard!$E$4:$K$4,0))</f>
         <v>25</v>
       </c>
       <c r="D12" s="10" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="33" t="n">
+      <c r="E12" s="10" t="n">
         <v>6</v>
       </c>
       <c r="F12" s="10" t="n">
@@ -3967,48 +4061,51 @@
       <c r="G12" s="10" t="n">
         <v>3.3</v>
       </c>
-      <c r="H12" s="36" t="n">
+      <c r="H12" s="37" t="n">
         <f aca="false">IF($E12&lt;2,"n/a",1-NORMDIST($C12,$F12,$G12,TRUE()))</f>
         <v>0.224352498756818</v>
       </c>
-      <c r="I12" s="37" t="n">
+      <c r="I12" s="38" t="n">
         <f aca="false">IF($E12&lt;2,"insufficient history",$C12*NORMDIST($C12,$F12,$G12,TRUE())+$F12*(1-NORMDIST($C12,$F12,$G12,TRUE()))+$G12*$G12*NORMDIST($C12,$F12,$G12,FALSE())-$C12)</f>
         <v>0.427213607902583</v>
       </c>
-      <c r="J12" s="38" t="str">
+      <c r="J12" s="39" t="str">
         <f aca="false">IF($E12&lt;2,"need &gt;=2 scores",IF($D12=0,"no attempts left",IF($I12&gt;=0.5,"SHOOT — best use of an attempt",IF($I12&gt;=0.15,"worthwhile","low return"))))</f>
         <v>worthwhile</v>
       </c>
-      <c r="K12" s="39" t="n">
+      <c r="K12" s="40" t="n">
         <f aca="false">IF(AND($D12&gt;0,$E12&gt;=2),$I12,-999)</f>
         <v>0.427213607902583</v>
       </c>
-      <c r="L12" s="40" t="str">
+      <c r="L12" s="41" t="str">
         <f aca="false">IF($E12&lt;2,"",REPT("|",ROUND(MAX($I12,0)*20,0)))</f>
         <v>|||||||||</v>
       </c>
+      <c r="N12" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="D14" s="41" t="str">
+        <v>127</v>
+      </c>
+      <c r="D14" s="42" t="str">
         <f aca="false">INDEX($B$6:$B$12,MATCH(MAX($K$6:$K$12),$K$6:$K$12,0))</f>
         <v>Mindsheets Masterpiece</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B15" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="C15" s="42"/>
-      <c r="D15" s="42"/>
-      <c r="E15" s="42"/>
-      <c r="F15" s="42"/>
-      <c r="G15" s="42"/>
-      <c r="H15" s="42"/>
-      <c r="I15" s="42"/>
-      <c r="J15" s="42"/>
+      <c r="B15" s="43" t="s">
+        <v>128</v>
+      </c>
+      <c r="C15" s="43"/>
+      <c r="D15" s="43"/>
+      <c r="E15" s="43"/>
+      <c r="F15" s="43"/>
+      <c r="G15" s="43"/>
+      <c r="H15" s="43"/>
+      <c r="I15" s="43"/>
+      <c r="J15" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>